<commit_message>
Areas of all foundations in all-footings.dxf
attached_areas.py now takes the DXF and output as arguments, adds the F2/F3
footings drawn in area 2, counts overlaps once and skips the duplicated
north-west raft polyline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/attached_areas.xlsx
+++ b/attached_areas.xlsx
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>209.61</v>
+        <v>209.42</v>
       </c>
       <c r="E20" t="n">
         <v>1120.9</v>
@@ -1087,7 +1087,7 @@
         <v>2.9</v>
       </c>
       <c r="H20" t="n">
-        <v>607.88</v>
+        <v>607.3200000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1117,13 +1117,13 @@
       </c>
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="n">
-        <v>209.61</v>
+        <v>209.42</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="n">
-        <v>607.88</v>
+        <v>607.3200000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1135,13 +1135,13 @@
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="n">
-        <v>1851.05</v>
+        <v>1850.86</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="n">
-        <v>4386.79</v>
+        <v>4386.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>